<commit_message>
Maximize EDGAR-sourced EV for backlog: fix EV gating, add net_debt, expand targeting
Three fixes so backlog EV comes from EDGAR wherever possible:
1. derived_ev was gated behind EBITDA>0 — but EV = mktCap + net debt and
   needs no EBITDA. Now computes whenever mktCap is derivable.
2. derived_net_debt now computed independently from EDGAR debt+cash facts
   (LongTermDebt + ShortTermBorrowings - Cash), not only when EBITDA exists.
3. Derive now targets ALL 1,332 backlog names (any region w/ CIK+price),
   not just US names missing PB/PE.

backfill_meta ev_total priority: explicit EV > SEC-derived EV > mktCap+net_debt.

Backlog EV coverage:
  net_debt from EDGAR:  676 → 1,320 / 1,332   (EV no longer understated)
  ev_total filled:      95% of backlog names
  backlog_to_ev:        1,239 names
  derived_ev overall:   478 → 1,549

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_016iHkWafvyERkeLmKLQn91d
</commit_message>
<xml_diff>
--- a/data/synthesis/workbook/archetypes_workbook_harvard.xlsx
+++ b/data/synthesis/workbook/archetypes_workbook_harvard.xlsx
@@ -14,12 +14,12 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="13133" uniqueCount="2505">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="13121" uniqueCount="2491">
   <si>
     <t>INVESTMENT ARCHETYPES  ·  CROSS-COHORT SUMMARY</t>
   </si>
   <si>
-    <t>2026-06-27  ·  18,680 ranked  ·  78 enduring  ·  97 turning  ·  509 cash  ·  277 segment-inflect  ·  246 backlog-inflect  ·  1554 triple-lens</t>
+    <t>2026-06-27  ·  18,680 ranked  ·  78 enduring  ·  97 turning  ·  509 cash  ·  277 segment-inflect  ·  246 backlog-inflect  ·  1556 triple-lens</t>
   </si>
   <si>
     <t>Each archetype is a structurally distinct setup. A name may appear in multiple cohorts — the Triple-Lens Conviction block at the end shows names with ≥ 3 archetype overlaps. Segment and backlog data come from full SEC EDGAR XBRL dimensional parsing (edgartools); fundamentals from Lindy multi-method ROIC reconciliation. Every cohort row shows the specific segment name, backlog concept, and inflection magnitude that drove the flag.</t>
@@ -1045,7 +1045,7 @@
     <t>Royalty</t>
   </si>
   <si>
-    <t>4. DEEP VALUE QUALITY — EV/EBIT ≤ 8 WITH ROIC ≥ 10 %  ·  108 NAMES</t>
+    <t>4. DEEP VALUE QUALITY — EV/EBIT ≤ 8 WITH ROIC ≥ 10 %  ·  110 NAMES</t>
   </si>
   <si>
     <t>THC</t>
@@ -2209,7 +2209,7 @@
     <t>NEOWIZ HOLDINDS</t>
   </si>
   <si>
-    <t>16. HIDDEN FCF GENERATORS — FCF MARGIN ≥ 10 % + EV/EBITDA ≤ 12  ·  76 NAMES</t>
+    <t>16. HIDDEN FCF GENERATORS — FCF MARGIN ≥ 10 % + EV/EBITDA ≤ 12  ·  79 NAMES</t>
   </si>
   <si>
     <t>FCAP</t>
@@ -2401,15 +2401,15 @@
     <t>Outside North Amer</t>
   </si>
   <si>
+    <t>FMCQF</t>
+  </si>
+  <si>
+    <t>Fresenius Medical Care AG</t>
+  </si>
+  <si>
     <t>FMS</t>
   </si>
   <si>
-    <t>Fresenius Medical Care AG</t>
-  </si>
-  <si>
-    <t>FMCQF</t>
-  </si>
-  <si>
     <t>17. REINVESTMENT HEROES — HIGH ROIIC + SIGNIFICANT CAPITAL DEPLOYMENT  ·  462 NAMES</t>
   </si>
   <si>
@@ -7237,7 +7237,7 @@
     <t>Scandinavian Investment Gr</t>
   </si>
   <si>
-    <t>24. SUB BOOK VALUE — GRAHAM DEEP VALUE (P/B &lt; 1)  ·  3988 NAMES</t>
+    <t>24. SUB BOOK VALUE — GRAHAM DEEP VALUE (P/B &lt; 1)  ·  3989 NAMES</t>
   </si>
   <si>
     <t>G0I.SI</t>
@@ -7414,7 +7414,7 @@
     <t>SILVER BULL RESOURCES INC</t>
   </si>
   <si>
-    <t>26. TRIPLE-LENS CONVICTION — PASSES ≥ 3 BUY-SIDE ARCHETYPES  ·  1554 NAMES</t>
+    <t>26. TRIPLE-LENS CONVICTION — PASSES ≥ 3 BUY-SIDE ARCHETYPES  ·  1556 NAMES</t>
   </si>
   <si>
     <t>Advanced Micro Devices, In</t>
@@ -7429,25 +7429,22 @@
     <t>CRESTEC INC</t>
   </si>
   <si>
-    <t>Investment Banking</t>
-  </si>
-  <si>
-    <t>ILMN</t>
-  </si>
-  <si>
-    <t>Illumina, Inc.</t>
-  </si>
-  <si>
-    <t>Sequencing</t>
-  </si>
-  <si>
-    <t>WTS</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Watts Water Technologies, </t>
-  </si>
-  <si>
-    <t>Specialty</t>
+    <t>General Dynamics Corporati</t>
+  </si>
+  <si>
+    <t>Contracts Accounte</t>
+  </si>
+  <si>
+    <t>7516.T</t>
+  </si>
+  <si>
+    <t>KOHNAN SHOJI</t>
+  </si>
+  <si>
+    <t>Modine Manufacturing Compa</t>
+  </si>
+  <si>
+    <t>Digital and Licens</t>
   </si>
   <si>
     <t>PFE</t>
@@ -7462,73 +7459,34 @@
     <t>Elrexfio</t>
   </si>
   <si>
-    <t>GDS.PA</t>
-  </si>
-  <si>
-    <t>RAMSAY GENERALE DE SANTE</t>
-  </si>
-  <si>
-    <t>EMN</t>
-  </si>
-  <si>
-    <t>Eastman Chemical Company</t>
-  </si>
-  <si>
-    <t>All Foreign Countr</t>
-  </si>
-  <si>
-    <t>Additives And Func</t>
-  </si>
-  <si>
-    <t>EHC</t>
-  </si>
-  <si>
-    <t>Encompass Health Corporati</t>
-  </si>
-  <si>
-    <t>Inpatient Rehabili</t>
-  </si>
-  <si>
-    <t>ORI</t>
-  </si>
-  <si>
-    <t>Old Republic International</t>
-  </si>
-  <si>
-    <t>GE</t>
-  </si>
-  <si>
-    <t>GE Aerospace</t>
-  </si>
-  <si>
-    <t>Equity method inve</t>
-  </si>
-  <si>
-    <t>PYPL</t>
-  </si>
-  <si>
-    <t>PayPal Holdings, Inc.</t>
-  </si>
-  <si>
-    <t>Transaction revenu</t>
-  </si>
-  <si>
-    <t>Revenues From Othe</t>
-  </si>
-  <si>
-    <t>Product and Servic</t>
-  </si>
-  <si>
-    <t>First Major Custom</t>
-  </si>
-  <si>
-    <t>8030.T</t>
-  </si>
-  <si>
-    <t>CHUO GYORUI CO LTD</t>
-  </si>
-  <si>
-    <t>L3Harris Technologies, Inc</t>
+    <t>NBIX</t>
+  </si>
+  <si>
+    <t>Neurocrine Biosciences, In</t>
+  </si>
+  <si>
+    <t>CRENESSITY net pro</t>
+  </si>
+  <si>
+    <t>7264.T</t>
+  </si>
+  <si>
+    <t>MURO CORPORATION</t>
+  </si>
+  <si>
+    <t>FFIV</t>
+  </si>
+  <si>
+    <t>F5, Inc.</t>
+  </si>
+  <si>
+    <t>Total Americas</t>
+  </si>
+  <si>
+    <t>JBI</t>
+  </si>
+  <si>
+    <t>Janus International Group,</t>
   </si>
 </sst>
 </file>
@@ -31848,7 +31806,7 @@
         <v>29</v>
       </c>
       <c r="E384" s="8">
-        <v>11623.477248</v>
+        <v>11279.715328</v>
       </c>
       <c r="F384" s="9">
         <v>9.84352572669953</v>
@@ -31863,10 +31821,10 @@
         <v>7.36287272875356</v>
       </c>
       <c r="J384" s="11">
-        <v>8.266542903324851</v>
+        <v>8.133928882692162</v>
       </c>
       <c r="K384" s="9">
-        <v>14.38746602517546</v>
+        <v>14.82594011791004</v>
       </c>
       <c r="L384" s="9">
         <v>-5.5</v>
@@ -31899,7 +31857,7 @@
         <v>30</v>
       </c>
       <c r="V384" s="11">
-        <v>69.4595824411135</v>
+        <v>71.07441113490363</v>
       </c>
     </row>
     <row r="385" spans="1:22">
@@ -31916,7 +31874,7 @@
         <v>29</v>
       </c>
       <c r="E385" s="8">
-        <v>11279.715328</v>
+        <v>11623.477248</v>
       </c>
       <c r="F385" s="9">
         <v>9.84352572669953</v>
@@ -31931,10 +31889,10 @@
         <v>7.36287272875356</v>
       </c>
       <c r="J385" s="11">
-        <v>8.133928882692162</v>
+        <v>8.266542903324851</v>
       </c>
       <c r="K385" s="9">
-        <v>14.82594011791004</v>
+        <v>14.38746602517546</v>
       </c>
       <c r="L385" s="9">
         <v>-5.5</v>
@@ -31967,7 +31925,7 @@
         <v>30</v>
       </c>
       <c r="V385" s="11">
-        <v>71.07441113490363</v>
+        <v>69.4595824411135</v>
       </c>
     </row>
     <row r="387" spans="1:22" ht="22" customHeight="1">
@@ -35211,8 +35169,8 @@
       <c r="T436" s="10" t="s">
         <v>30</v>
       </c>
-      <c r="U436" s="10" t="s">
-        <v>30</v>
+      <c r="U436" s="11">
+        <v>18.27730411367763</v>
       </c>
       <c r="V436" s="11">
         <v>70.76231263383298</v>
@@ -43575,8 +43533,8 @@
       <c r="T559" s="10" t="s">
         <v>30</v>
       </c>
-      <c r="U559" s="10" t="s">
-        <v>30</v>
+      <c r="U559" s="11">
+        <v>11.69403989340236</v>
       </c>
       <c r="V559" s="11">
         <v>75.69111349036403</v>
@@ -59046,10 +59004,10 @@
         <v>30</v>
       </c>
       <c r="O790" s="8">
-        <v>3593.527898567871</v>
+        <v>3415.832898567871</v>
       </c>
       <c r="P790" s="11">
-        <v>0.0011498449759209</v>
+        <v>0.0012096610468657</v>
       </c>
       <c r="Q790" s="9">
         <v>-7.923636466348261</v>
@@ -59114,10 +59072,10 @@
         <v>30</v>
       </c>
       <c r="O791" s="8">
-        <v>2045.064322196083</v>
+        <v>2016.193322196083</v>
       </c>
       <c r="P791" s="11">
-        <v>0.0008801679147514</v>
+        <v>0.0008927715314716</v>
       </c>
       <c r="Q791" s="9">
         <v>-28.90813072165297</v>
@@ -59182,10 +59140,10 @@
         <v>0.0534529753720722</v>
       </c>
       <c r="O792" s="8">
-        <v>308.4474645</v>
+        <v>298.6534645</v>
       </c>
       <c r="P792" s="11">
-        <v>0.0071843676964314</v>
+        <v>0.0074199708471823</v>
       </c>
       <c r="Q792" s="9">
         <v>5.05593634957493</v>
@@ -59250,10 +59208,10 @@
         <v>0.4801656793921028</v>
       </c>
       <c r="O793" s="8">
-        <v>98.13520722165775</v>
+        <v>146.1832072216578</v>
       </c>
       <c r="P793" s="11">
-        <v>0.6426235984559292</v>
+        <v>0.4314038609398957</v>
       </c>
       <c r="Q793" s="9">
         <v>5.31940257538757</v>
@@ -59386,10 +59344,10 @@
         <v>9.229655872631827E-06</v>
       </c>
       <c r="O795" s="8">
-        <v>58.82066565805078</v>
+        <v>63.23466565805077</v>
       </c>
       <c r="P795" s="11">
-        <v>2.905441447968533E-05</v>
+        <v>2.702631511079109E-05</v>
       </c>
       <c r="Q795" s="9">
         <v>-14.94478982766374</v>
@@ -59454,10 +59412,10 @@
         <v>30</v>
       </c>
       <c r="O796" s="8">
-        <v>28.99893278182984</v>
+        <v>32.50425478182984</v>
       </c>
       <c r="P796" s="11">
-        <v>0.0015354013313172</v>
+        <v>0.0013698206680588</v>
       </c>
       <c r="Q796" s="9">
         <v>-192.9559070228838</v>
@@ -59522,10 +59480,10 @@
         <v>30</v>
       </c>
       <c r="O797" s="8">
-        <v>1860.478791775177</v>
+        <v>1703.101791775177</v>
       </c>
       <c r="P797" s="11">
-        <v>0.0026874802454637</v>
+        <v>0.002935819822483</v>
       </c>
       <c r="Q797" s="9">
         <v>4.09292371790951</v>
@@ -59726,10 +59684,10 @@
         <v>0.1821366024518388</v>
       </c>
       <c r="O800" s="8">
-        <v>24.43764225</v>
+        <v>24.20564725</v>
       </c>
       <c r="P800" s="11">
-        <v>0.0085114594064408</v>
+        <v>0.0085930360734311</v>
       </c>
       <c r="Q800" s="9">
         <v>-84.36971799652343</v>
@@ -59794,7 +59752,7 @@
         <v>30</v>
       </c>
       <c r="O801" s="8">
-        <v>174.1593132094502</v>
+        <v>85.55931320945024</v>
       </c>
       <c r="P801" s="11">
         <v>0</v>
@@ -59862,10 +59820,10 @@
         <v>30</v>
       </c>
       <c r="O802" s="8">
-        <v>11.49093503085476</v>
+        <v>11.35593503085476</v>
       </c>
       <c r="P802" s="11">
-        <v>0.0363765001610062</v>
+        <v>0.0368089460589787</v>
       </c>
       <c r="Q802" s="9">
         <v>-23.4322448250743</v>
@@ -59930,10 +59888,10 @@
         <v>0.0077674883923761</v>
       </c>
       <c r="O803" s="8">
-        <v>121.6679051485062</v>
+        <v>124.6889051485062</v>
       </c>
       <c r="P803" s="11">
-        <v>0.0248874178963142</v>
+        <v>0.0242844381093378</v>
       </c>
       <c r="Q803" s="9">
         <v>5.50919798972899</v>
@@ -59998,10 +59956,10 @@
         <v>30</v>
       </c>
       <c r="O804" s="8">
-        <v>90.87370453641176</v>
+        <v>83.32959753641177</v>
       </c>
       <c r="P804" s="11">
-        <v>0.0021853626526299</v>
+        <v>0.0023832108383005</v>
       </c>
       <c r="Q804" s="9">
         <v>-39.87834427298205</v>
@@ -60066,10 +60024,10 @@
         <v>0.1349228890864358</v>
       </c>
       <c r="O805" s="8">
-        <v>478.8987191348124</v>
+        <v>407.2467191348124</v>
       </c>
       <c r="P805" s="11">
-        <v>0.0763794066229337</v>
+        <v>0.08981778926963301</v>
       </c>
       <c r="Q805" s="9">
         <v>-27.68875261121275</v>
@@ -60134,10 +60092,10 @@
         <v>30</v>
       </c>
       <c r="O806" s="8">
-        <v>3561.385401522064</v>
+        <v>6168.685401522064</v>
       </c>
       <c r="P806" s="11">
-        <v>0.0192060089791931</v>
+        <v>0.0110882620117282</v>
       </c>
       <c r="Q806" s="9">
         <v>2.66863929893312</v>
@@ -60202,10 +60160,10 @@
         <v>30</v>
       </c>
       <c r="O807" s="8">
-        <v>48.97052133011818</v>
+        <v>88.19952133011817</v>
       </c>
       <c r="P807" s="11">
-        <v>0.2153744684256263</v>
+        <v>0.1195811478446021</v>
       </c>
       <c r="Q807" s="9">
         <v>-5.53381200735645</v>
@@ -60270,10 +60228,10 @@
         <v>0.1079811973656467</v>
       </c>
       <c r="O808" s="8">
-        <v>86.06846457688617</v>
-      </c>
-      <c r="P808" s="11">
-        <v>0.5057717738314379</v>
+        <v>-80.76153542311383</v>
+      </c>
+      <c r="P808" s="10" t="s">
+        <v>30</v>
       </c>
       <c r="Q808" s="9">
         <v>-30.9163890684529</v>
@@ -60338,10 +60296,10 @@
         <v>30</v>
       </c>
       <c r="O809" s="8">
-        <v>488.6488407275962</v>
+        <v>482.5738407275962</v>
       </c>
       <c r="P809" s="11">
-        <v>0.0008574664771047</v>
+        <v>0.0008682609056642</v>
       </c>
       <c r="Q809" s="9">
         <v>-27.64249887755216</v>
@@ -60474,7 +60432,7 @@
         <v>30</v>
       </c>
       <c r="O811" s="8">
-        <v>2911.235683953965</v>
+        <v>2705.909683953965</v>
       </c>
       <c r="P811" s="11">
         <v>0</v>
@@ -60610,10 +60568,10 @@
         <v>0.050581338833265</v>
       </c>
       <c r="O813" s="8">
-        <v>2244.875886780533</v>
+        <v>1882.757886780533</v>
       </c>
       <c r="P813" s="11">
-        <v>0.04798127176397</v>
+        <v>0.0572096926303066</v>
       </c>
       <c r="Q813" s="9">
         <v>38.76866695640053</v>
@@ -60678,10 +60636,10 @@
         <v>0.0210824130692707</v>
       </c>
       <c r="O814" s="8">
-        <v>110.1124877091591</v>
+        <v>301.2234877091591</v>
       </c>
       <c r="P814" s="11">
-        <v>0.0188806923106784</v>
+        <v>0.0069018522287589</v>
       </c>
       <c r="Q814" s="9">
         <v>-7.002080052003739</v>
@@ -60746,10 +60704,10 @@
         <v>0.0557043385109801</v>
       </c>
       <c r="O815" s="8">
-        <v>3835.6261369468</v>
+        <v>4836.6261369468</v>
       </c>
       <c r="P815" s="11">
-        <v>0.0271142171543301</v>
+        <v>0.0215025923144127</v>
       </c>
       <c r="Q815" s="9">
         <v>2.07805985698824</v>
@@ -60814,10 +60772,10 @@
         <v>30</v>
       </c>
       <c r="O816" s="8">
-        <v>39.76181969904901</v>
+        <v>89.790819699049</v>
       </c>
       <c r="P816" s="11">
-        <v>0.2187525637869142</v>
+        <v>0.0968695912249492</v>
       </c>
       <c r="Q816" s="9">
         <v>-5.34485212061657</v>
@@ -61086,10 +61044,10 @@
         <v>0.0382982588989762</v>
       </c>
       <c r="O820" s="8">
-        <v>10995.61919360275</v>
+        <v>11011.60619360275</v>
       </c>
       <c r="P820" s="11">
-        <v>0.0050228185450558</v>
+        <v>0.0050155262573851</v>
       </c>
       <c r="Q820" s="9">
         <v>17.79581484188693</v>
@@ -61222,10 +61180,10 @@
         <v>30</v>
       </c>
       <c r="O822" s="8">
-        <v>51.97174673283005</v>
+        <v>165.59443673283</v>
       </c>
       <c r="P822" s="11">
-        <v>0.470024610209398</v>
+        <v>0.1475170330716612</v>
       </c>
       <c r="Q822" s="9">
         <v>-0.24148789738567</v>
@@ -61290,10 +61248,10 @@
         <v>30</v>
       </c>
       <c r="O823" s="8">
-        <v>60.26884763805008</v>
+        <v>173.8915376380501</v>
       </c>
       <c r="P823" s="11">
-        <v>0.4053171905111663</v>
+        <v>0.1404783713560928</v>
       </c>
       <c r="Q823" s="9">
         <v>-0.24148789738567</v>
@@ -61630,10 +61588,10 @@
         <v>30</v>
       </c>
       <c r="O828" s="8">
-        <v>107.931804</v>
+        <v>103.473736</v>
       </c>
       <c r="P828" s="11">
-        <v>0.0041746638460708</v>
+        <v>0.0043545252874603</v>
       </c>
       <c r="Q828" s="9">
         <v>0.18734908473256</v>
@@ -63189,8 +63147,8 @@
       <c r="D853" s="7" t="s">
         <v>29</v>
       </c>
-      <c r="E853" s="10" t="s">
-        <v>30</v>
+      <c r="E853" s="8">
+        <v>55444.61966705322</v>
       </c>
       <c r="F853" s="9">
         <v>2.87828660024318</v>
@@ -70720,61 +70678,61 @@
     </row>
     <row r="972" spans="1:22">
       <c r="A972" s="6" t="s">
-        <v>130</v>
+        <v>1459</v>
       </c>
       <c r="B972" s="7" t="s">
-        <v>131</v>
+        <v>1460</v>
       </c>
       <c r="C972" s="7" t="s">
         <v>28</v>
       </c>
       <c r="D972" s="7" t="s">
-        <v>49</v>
+        <v>29</v>
       </c>
       <c r="E972" s="8">
-        <v>3569.760046005249</v>
+        <v>23249.096704</v>
       </c>
       <c r="F972" s="9">
-        <v>44.56422400643385</v>
+        <v>10.58799092293385</v>
       </c>
       <c r="G972" s="9">
-        <v>39.32576921819311</v>
-      </c>
-      <c r="H972" s="10" t="s">
-        <v>30</v>
+        <v>-0.28771197424686</v>
+      </c>
+      <c r="H972" s="9">
+        <v>-28.16427067427359</v>
       </c>
       <c r="I972" s="9">
-        <v>44.16783713667234</v>
+        <v>15.2922875171542</v>
       </c>
       <c r="J972" s="11">
-        <v>4.12189438130252</v>
-      </c>
-      <c r="K972" s="10" t="s">
-        <v>30</v>
-      </c>
-      <c r="L972" s="10" t="s">
-        <v>30</v>
+        <v>7.34889280734496</v>
+      </c>
+      <c r="K972" s="9">
+        <v>-4.3921347181816</v>
+      </c>
+      <c r="L972" s="9">
+        <v>-16.9</v>
       </c>
       <c r="M972" s="7" t="s">
-        <v>132</v>
+        <v>246</v>
       </c>
       <c r="N972" s="9">
-        <v>69.19229807451863</v>
+        <v>83.23873211902226</v>
       </c>
       <c r="O972" s="7" t="s">
-        <v>132</v>
+        <v>1462</v>
       </c>
       <c r="P972" s="9">
-        <v>0.4902850917014811</v>
+        <v>66.5089585090408</v>
       </c>
       <c r="Q972" s="9">
-        <v>1.638323589729629</v>
-      </c>
-      <c r="R972" s="7" t="s">
-        <v>46</v>
-      </c>
-      <c r="S972" s="9">
-        <v>10.69455163709715</v>
+        <v>61.17457010769595</v>
+      </c>
+      <c r="R972" s="10" t="s">
+        <v>30</v>
+      </c>
+      <c r="S972" s="10" t="s">
+        <v>30</v>
       </c>
       <c r="T972" s="10" t="s">
         <v>30</v>
@@ -70783,151 +70741,151 @@
         <v>41</v>
       </c>
       <c r="V972" s="11">
-        <v>26.81986081370449</v>
+        <v>47.91327623126338</v>
       </c>
     </row>
     <row r="973" spans="1:22">
       <c r="A973" s="6" t="s">
-        <v>1083</v>
+        <v>130</v>
       </c>
       <c r="B973" s="7" t="s">
-        <v>2467</v>
+        <v>131</v>
       </c>
       <c r="C973" s="7" t="s">
         <v>28</v>
       </c>
       <c r="D973" s="7" t="s">
-        <v>106</v>
+        <v>49</v>
       </c>
       <c r="E973" s="8">
-        <v>762322.092032</v>
+        <v>3569.760046005249</v>
       </c>
       <c r="F973" s="9">
-        <v>14.39909228246559</v>
+        <v>44.56422400643385</v>
       </c>
       <c r="G973" s="9">
-        <v>0.76076645797761</v>
-      </c>
-      <c r="H973" s="9">
-        <v>47.26579989976284</v>
+        <v>39.32576921819311</v>
+      </c>
+      <c r="H973" s="10" t="s">
+        <v>30</v>
       </c>
       <c r="I973" s="9">
-        <v>17.08548321355481</v>
+        <v>44.16783713667234</v>
       </c>
       <c r="J973" s="11">
-        <v>101.4597684119986</v>
-      </c>
-      <c r="K973" s="9">
-        <v>0.94099004226403</v>
-      </c>
-      <c r="L973" s="9">
-        <v>37.8</v>
+        <v>4.12189438130252</v>
+      </c>
+      <c r="K973" s="10" t="s">
+        <v>30</v>
+      </c>
+      <c r="L973" s="10" t="s">
+        <v>30</v>
       </c>
       <c r="M973" s="7" t="s">
-        <v>197</v>
+        <v>132</v>
       </c>
       <c r="N973" s="9">
-        <v>24.53293446971835</v>
+        <v>69.19229807451863</v>
       </c>
       <c r="O973" s="7" t="s">
-        <v>1085</v>
+        <v>132</v>
       </c>
       <c r="P973" s="9">
-        <v>467.7697841726618</v>
+        <v>0.4902850917014811</v>
       </c>
       <c r="Q973" s="9">
-        <v>10.34555214833951</v>
+        <v>1.638323589729629</v>
       </c>
       <c r="R973" s="7" t="s">
-        <v>52</v>
+        <v>46</v>
       </c>
       <c r="S973" s="9">
-        <v>178.9746882258184</v>
-      </c>
-      <c r="T973" s="12" t="s">
-        <v>41</v>
+        <v>10.69455163709715</v>
+      </c>
+      <c r="T973" s="10" t="s">
+        <v>30</v>
       </c>
       <c r="U973" s="12" t="s">
         <v>41</v>
       </c>
       <c r="V973" s="11">
-        <v>56.21306209850107</v>
+        <v>26.81986081370449</v>
       </c>
     </row>
     <row r="974" spans="1:22">
       <c r="A974" s="6" t="s">
-        <v>1459</v>
+        <v>1083</v>
       </c>
       <c r="B974" s="7" t="s">
-        <v>1460</v>
+        <v>2467</v>
       </c>
       <c r="C974" s="7" t="s">
         <v>28</v>
       </c>
       <c r="D974" s="7" t="s">
-        <v>29</v>
+        <v>106</v>
       </c>
       <c r="E974" s="8">
-        <v>23249.096704</v>
+        <v>762322.092032</v>
       </c>
       <c r="F974" s="9">
-        <v>10.58799092293385</v>
+        <v>14.39909228246559</v>
       </c>
       <c r="G974" s="9">
-        <v>-0.28771197424686</v>
+        <v>0.76076645797761</v>
       </c>
       <c r="H974" s="9">
-        <v>-28.16427067427359</v>
+        <v>47.26579989976284</v>
       </c>
       <c r="I974" s="9">
-        <v>15.2922875171542</v>
+        <v>17.08548321355481</v>
       </c>
       <c r="J974" s="11">
-        <v>7.34889280734496</v>
+        <v>101.4597684119986</v>
       </c>
       <c r="K974" s="9">
-        <v>-4.3921347181816</v>
+        <v>0.94099004226403</v>
       </c>
       <c r="L974" s="9">
-        <v>-16.9</v>
+        <v>37.8</v>
       </c>
       <c r="M974" s="7" t="s">
-        <v>246</v>
+        <v>197</v>
       </c>
       <c r="N974" s="9">
-        <v>83.23873211902226</v>
+        <v>24.53293446971835</v>
       </c>
       <c r="O974" s="7" t="s">
-        <v>1462</v>
+        <v>1085</v>
       </c>
       <c r="P974" s="9">
-        <v>66.5089585090408</v>
+        <v>467.7697841726618</v>
       </c>
       <c r="Q974" s="9">
-        <v>61.17457010769595</v>
-      </c>
-      <c r="R974" s="10" t="s">
-        <v>30</v>
-      </c>
-      <c r="S974" s="10" t="s">
-        <v>30</v>
-      </c>
-      <c r="T974" s="10" t="s">
-        <v>30</v>
+        <v>10.34555214833951</v>
+      </c>
+      <c r="R974" s="7" t="s">
+        <v>52</v>
+      </c>
+      <c r="S974" s="9">
+        <v>178.9746882258184</v>
+      </c>
+      <c r="T974" s="12" t="s">
+        <v>41</v>
       </c>
       <c r="U974" s="12" t="s">
         <v>41</v>
       </c>
       <c r="V974" s="11">
-        <v>47.91327623126338</v>
+        <v>56.21306209850107</v>
       </c>
     </row>
     <row r="975" spans="1:22">
       <c r="A975" s="6" t="s">
-        <v>786</v>
+        <v>1701</v>
       </c>
       <c r="B975" s="7" t="s">
-        <v>787</v>
+        <v>1702</v>
       </c>
       <c r="C975" s="7" t="s">
         <v>28</v>
@@ -70936,126 +70894,126 @@
         <v>29</v>
       </c>
       <c r="E975" s="8">
-        <v>12134.3232</v>
+        <v>12578.661376</v>
       </c>
       <c r="F975" s="9">
-        <v>14.03638757502264</v>
+        <v>20.21134884265646</v>
       </c>
       <c r="G975" s="9">
-        <v>6.90913608330241</v>
+        <v>16.4350192965183</v>
       </c>
       <c r="H975" s="9">
-        <v>15.9424688855513</v>
+        <v>-39.21585735433231</v>
       </c>
       <c r="I975" s="9">
-        <v>21.17626443534281</v>
+        <v>20.9006052706891</v>
       </c>
       <c r="J975" s="11">
-        <v>9.129744194863251</v>
-      </c>
-      <c r="K975" s="9">
-        <v>10.85536511834463</v>
+        <v>7.88744587549017</v>
+      </c>
+      <c r="K975" s="10" t="s">
+        <v>30</v>
       </c>
       <c r="L975" s="9">
-        <v>5.4</v>
+        <v>-7.6</v>
       </c>
       <c r="M975" s="7" t="s">
-        <v>81</v>
+        <v>1703</v>
       </c>
       <c r="N975" s="9">
-        <v>100</v>
+        <v>53.42455018949013</v>
       </c>
       <c r="O975" s="7" t="s">
-        <v>81</v>
+        <v>2468</v>
       </c>
       <c r="P975" s="9">
-        <v>-8.981387797359941</v>
+        <v>26.88567771615129</v>
       </c>
       <c r="Q975" s="9">
-        <v>0</v>
-      </c>
-      <c r="R975" s="10" t="s">
-        <v>30</v>
-      </c>
-      <c r="S975" s="10" t="s">
-        <v>30</v>
+        <v>46.64781228573134</v>
+      </c>
+      <c r="R975" s="7" t="s">
+        <v>46</v>
+      </c>
+      <c r="S975" s="9">
+        <v>-185.986970028494</v>
       </c>
       <c r="T975" s="10" t="s">
         <v>30</v>
       </c>
-      <c r="U975" s="10" t="s">
-        <v>30</v>
+      <c r="U975" s="12" t="s">
+        <v>41</v>
       </c>
       <c r="V975" s="11">
-        <v>78.19432548179871</v>
+        <v>44.63811563169165</v>
       </c>
     </row>
     <row r="976" spans="1:22">
       <c r="A976" s="6" t="s">
-        <v>1701</v>
+        <v>2469</v>
       </c>
       <c r="B976" s="7" t="s">
-        <v>1702</v>
+        <v>2470</v>
       </c>
       <c r="C976" s="7" t="s">
-        <v>28</v>
+        <v>431</v>
       </c>
       <c r="D976" s="7" t="s">
-        <v>29</v>
+        <v>275</v>
       </c>
       <c r="E976" s="8">
-        <v>12578.661376</v>
-      </c>
-      <c r="F976" s="9">
-        <v>20.21134884265646</v>
-      </c>
-      <c r="G976" s="9">
-        <v>16.4350192965183</v>
-      </c>
-      <c r="H976" s="9">
-        <v>-39.21585735433231</v>
-      </c>
-      <c r="I976" s="9">
-        <v>20.9006052706891</v>
+        <v>5982.524928</v>
+      </c>
+      <c r="F976" s="10" t="s">
+        <v>30</v>
+      </c>
+      <c r="G976" s="10" t="s">
+        <v>30</v>
+      </c>
+      <c r="H976" s="10" t="s">
+        <v>30</v>
+      </c>
+      <c r="I976" s="10" t="s">
+        <v>30</v>
       </c>
       <c r="J976" s="11">
-        <v>7.88744587549017</v>
+        <v>2.384461875584978</v>
       </c>
       <c r="K976" s="10" t="s">
         <v>30</v>
       </c>
       <c r="L976" s="9">
-        <v>-7.6</v>
-      </c>
-      <c r="M976" s="7" t="s">
-        <v>1703</v>
-      </c>
-      <c r="N976" s="9">
-        <v>53.42455018949013</v>
-      </c>
-      <c r="O976" s="7" t="s">
-        <v>2468</v>
-      </c>
-      <c r="P976" s="9">
-        <v>26.88567771615129</v>
-      </c>
-      <c r="Q976" s="9">
-        <v>46.64781228573134</v>
-      </c>
-      <c r="R976" s="7" t="s">
-        <v>46</v>
-      </c>
-      <c r="S976" s="9">
-        <v>-185.986970028494</v>
+        <v>-2.6</v>
+      </c>
+      <c r="M976" s="10" t="s">
+        <v>30</v>
+      </c>
+      <c r="N976" s="10" t="s">
+        <v>30</v>
+      </c>
+      <c r="O976" s="10" t="s">
+        <v>30</v>
+      </c>
+      <c r="P976" s="10" t="s">
+        <v>30</v>
+      </c>
+      <c r="Q976" s="10" t="s">
+        <v>30</v>
+      </c>
+      <c r="R976" s="10" t="s">
+        <v>30</v>
+      </c>
+      <c r="S976" s="10" t="s">
+        <v>30</v>
       </c>
       <c r="T976" s="10" t="s">
         <v>30</v>
       </c>
-      <c r="U976" s="12" t="s">
-        <v>41</v>
+      <c r="U976" s="10" t="s">
+        <v>30</v>
       </c>
       <c r="V976" s="11">
-        <v>44.63811563169165</v>
+        <v>80.55594218415418</v>
       </c>
     </row>
     <row r="977" spans="1:22">
@@ -71128,55 +71086,55 @@
     </row>
     <row r="978" spans="1:22">
       <c r="A978" s="6" t="s">
-        <v>2469</v>
+        <v>212</v>
       </c>
       <c r="B978" s="7" t="s">
-        <v>2470</v>
+        <v>213</v>
       </c>
       <c r="C978" s="7" t="s">
-        <v>431</v>
+        <v>28</v>
       </c>
       <c r="D978" s="7" t="s">
-        <v>275</v>
+        <v>106</v>
       </c>
       <c r="E978" s="8">
-        <v>5982.524928</v>
-      </c>
-      <c r="F978" s="10" t="s">
-        <v>30</v>
-      </c>
-      <c r="G978" s="10" t="s">
-        <v>30</v>
-      </c>
-      <c r="H978" s="10" t="s">
-        <v>30</v>
-      </c>
-      <c r="I978" s="10" t="s">
-        <v>30</v>
+        <v>564107.214848</v>
+      </c>
+      <c r="F978" s="9">
+        <v>25.37691905817877</v>
+      </c>
+      <c r="G978" s="9">
+        <v>22.23484640325328</v>
+      </c>
+      <c r="H978" s="9">
+        <v>460.1372328458942</v>
+      </c>
+      <c r="I978" s="9">
+        <v>25.4315100204583</v>
       </c>
       <c r="J978" s="11">
-        <v>2.384461875584978</v>
-      </c>
-      <c r="K978" s="10" t="s">
-        <v>30</v>
+        <v>17.39382995030982</v>
+      </c>
+      <c r="K978" s="9">
+        <v>2.21790734645562</v>
       </c>
       <c r="L978" s="9">
-        <v>-2.6</v>
-      </c>
-      <c r="M978" s="10" t="s">
-        <v>30</v>
-      </c>
-      <c r="N978" s="10" t="s">
-        <v>30</v>
-      </c>
-      <c r="O978" s="10" t="s">
-        <v>30</v>
-      </c>
-      <c r="P978" s="10" t="s">
-        <v>30</v>
-      </c>
-      <c r="Q978" s="10" t="s">
-        <v>30</v>
+        <v>9.9</v>
+      </c>
+      <c r="M978" s="7" t="s">
+        <v>214</v>
+      </c>
+      <c r="N978" s="9">
+        <v>21.37774708778672</v>
+      </c>
+      <c r="O978" s="7" t="s">
+        <v>215</v>
+      </c>
+      <c r="P978" s="9">
+        <v>355.5555555555555</v>
+      </c>
+      <c r="Q978" s="9">
+        <v>0.7092925360709185</v>
       </c>
       <c r="R978" s="10" t="s">
         <v>30</v>
@@ -71184,67 +71142,67 @@
       <c r="S978" s="10" t="s">
         <v>30</v>
       </c>
-      <c r="T978" s="10" t="s">
-        <v>30</v>
-      </c>
-      <c r="U978" s="10" t="s">
-        <v>30</v>
+      <c r="T978" s="12" t="s">
+        <v>41</v>
+      </c>
+      <c r="U978" s="12" t="s">
+        <v>41</v>
       </c>
       <c r="V978" s="11">
-        <v>80.55594218415418</v>
+        <v>38.20824411134903</v>
       </c>
     </row>
     <row r="979" spans="1:22">
       <c r="A979" s="6" t="s">
-        <v>212</v>
+        <v>786</v>
       </c>
       <c r="B979" s="7" t="s">
-        <v>213</v>
+        <v>787</v>
       </c>
       <c r="C979" s="7" t="s">
         <v>28</v>
       </c>
       <c r="D979" s="7" t="s">
-        <v>106</v>
+        <v>29</v>
       </c>
       <c r="E979" s="8">
-        <v>564107.214848</v>
+        <v>12134.3232</v>
       </c>
       <c r="F979" s="9">
-        <v>25.37691905817877</v>
+        <v>14.03638757502264</v>
       </c>
       <c r="G979" s="9">
-        <v>22.23484640325328</v>
+        <v>6.90913608330241</v>
       </c>
       <c r="H979" s="9">
-        <v>460.1372328458942</v>
+        <v>15.9424688855513</v>
       </c>
       <c r="I979" s="9">
-        <v>25.4315100204583</v>
+        <v>21.17626443534281</v>
       </c>
       <c r="J979" s="11">
-        <v>17.39382995030982</v>
+        <v>9.129744194863251</v>
       </c>
       <c r="K979" s="9">
-        <v>2.21790734645562</v>
+        <v>10.85536511834463</v>
       </c>
       <c r="L979" s="9">
-        <v>9.9</v>
+        <v>5.4</v>
       </c>
       <c r="M979" s="7" t="s">
-        <v>214</v>
+        <v>81</v>
       </c>
       <c r="N979" s="9">
-        <v>21.37774708778672</v>
+        <v>100</v>
       </c>
       <c r="O979" s="7" t="s">
-        <v>215</v>
+        <v>81</v>
       </c>
       <c r="P979" s="9">
-        <v>355.5555555555555</v>
+        <v>-8.981387797359941</v>
       </c>
       <c r="Q979" s="9">
-        <v>0.7092925360709185</v>
+        <v>0</v>
       </c>
       <c r="R979" s="10" t="s">
         <v>30</v>
@@ -71252,22 +71210,22 @@
       <c r="S979" s="10" t="s">
         <v>30</v>
       </c>
-      <c r="T979" s="12" t="s">
-        <v>41</v>
-      </c>
-      <c r="U979" s="12" t="s">
-        <v>41</v>
+      <c r="T979" s="10" t="s">
+        <v>30</v>
+      </c>
+      <c r="U979" s="10" t="s">
+        <v>30</v>
       </c>
       <c r="V979" s="11">
-        <v>38.20824411134903</v>
+        <v>78.19432548179871</v>
       </c>
     </row>
     <row r="980" spans="1:22">
       <c r="A980" s="6" t="s">
-        <v>2049</v>
+        <v>1986</v>
       </c>
       <c r="B980" s="7" t="s">
-        <v>2050</v>
+        <v>2471</v>
       </c>
       <c r="C980" s="7" t="s">
         <v>28</v>
@@ -71276,117 +71234,117 @@
         <v>29</v>
       </c>
       <c r="E980" s="8">
-        <v>13388.781568</v>
+        <v>92727.803904</v>
       </c>
       <c r="F980" s="9">
-        <v>36.47155849611668</v>
+        <v>12.16832467586076</v>
       </c>
       <c r="G980" s="9">
-        <v>19.02096509492922</v>
+        <v>11.8119306083982</v>
       </c>
       <c r="H980" s="9">
-        <v>200</v>
-      </c>
-      <c r="I980" s="10" t="s">
-        <v>30</v>
-      </c>
-      <c r="J980" s="10" t="s">
-        <v>30</v>
-      </c>
-      <c r="K980" s="10" t="s">
-        <v>30</v>
+        <v>25.2816769962534</v>
+      </c>
+      <c r="I980" s="9">
+        <v>11.87076192256857</v>
+      </c>
+      <c r="J980" s="11">
+        <v>15.2467708167422</v>
+      </c>
+      <c r="K980" s="9">
+        <v>5.70433024109592</v>
       </c>
       <c r="L980" s="9">
-        <v>100.3</v>
+        <v>10.3</v>
       </c>
       <c r="M980" s="7" t="s">
-        <v>2471</v>
+        <v>1988</v>
       </c>
       <c r="N980" s="9">
-        <v>48.14443778928729</v>
+        <v>12.7768650489863</v>
       </c>
       <c r="O980" s="7" t="s">
-        <v>2052</v>
+        <v>2472</v>
       </c>
       <c r="P980" s="9">
-        <v>33.86381655368238</v>
+        <v>71.59090909090908</v>
       </c>
       <c r="Q980" s="9">
-        <v>1.118296032840677</v>
+        <v>1.149159869153103</v>
       </c>
       <c r="R980" s="7" t="s">
-        <v>46</v>
-      </c>
-      <c r="S980" s="9">
-        <v>139.17336501721</v>
+        <v>52</v>
+      </c>
+      <c r="S980" s="10" t="s">
+        <v>30</v>
       </c>
       <c r="T980" s="10" t="s">
         <v>30</v>
       </c>
-      <c r="U980" s="10" t="s">
-        <v>30</v>
+      <c r="U980" s="12" t="s">
+        <v>41</v>
       </c>
       <c r="V980" s="11">
-        <v>53.42826552462527</v>
+        <v>67.19860813704497</v>
       </c>
     </row>
     <row r="981" spans="1:22">
       <c r="A981" s="6" t="s">
-        <v>2472</v>
+        <v>174</v>
       </c>
       <c r="B981" s="7" t="s">
-        <v>2473</v>
+        <v>175</v>
       </c>
       <c r="C981" s="7" t="s">
         <v>28</v>
       </c>
       <c r="D981" s="7" t="s">
-        <v>29</v>
+        <v>106</v>
       </c>
       <c r="E981" s="8">
-        <v>21849.233408</v>
+        <v>456181.284864</v>
       </c>
       <c r="F981" s="9">
-        <v>-11.74199733282329</v>
+        <v>30.37976197045843</v>
       </c>
       <c r="G981" s="9">
-        <v>-38.48741508262834</v>
+        <v>27.99861973775017</v>
       </c>
       <c r="H981" s="9">
-        <v>368.4856669297553</v>
+        <v>58.3123045780253</v>
       </c>
       <c r="I981" s="9">
-        <v>14.7476304816127</v>
+        <v>46.45975544187588</v>
       </c>
       <c r="J981" s="11">
-        <v>20.11968143406094</v>
+        <v>33.82491037527318</v>
       </c>
       <c r="K981" s="9">
-        <v>3.87027319544482</v>
+        <v>1.46660448159213</v>
       </c>
       <c r="L981" s="9">
-        <v>4.8</v>
+        <v>21.5</v>
       </c>
       <c r="M981" s="7" t="s">
-        <v>2474</v>
+        <v>176</v>
       </c>
       <c r="N981" s="9">
-        <v>20.94963273871983</v>
+        <v>49.52110586060094</v>
       </c>
       <c r="O981" s="7" t="s">
-        <v>1066</v>
+        <v>177</v>
       </c>
       <c r="P981" s="9">
-        <v>3.947368421052633</v>
+        <v>7.014416611939822</v>
       </c>
       <c r="Q981" s="9">
-        <v>1.223071606310058</v>
+        <v>0.1267569180761707</v>
       </c>
       <c r="R981" s="7" t="s">
-        <v>52</v>
-      </c>
-      <c r="S981" s="9">
-        <v>7.556287570432973</v>
+        <v>139</v>
+      </c>
+      <c r="S981" s="10" t="s">
+        <v>30</v>
       </c>
       <c r="T981" s="12" t="s">
         <v>41</v>
@@ -71395,66 +71353,66 @@
         <v>30</v>
       </c>
       <c r="V981" s="11">
-        <v>65.34716274089935</v>
+        <v>71.76472162740899</v>
       </c>
     </row>
     <row r="982" spans="1:22">
       <c r="A982" s="6" t="s">
-        <v>2475</v>
+        <v>2004</v>
       </c>
       <c r="B982" s="7" t="s">
-        <v>2476</v>
+        <v>2005</v>
       </c>
       <c r="C982" s="7" t="s">
         <v>28</v>
       </c>
       <c r="D982" s="7" t="s">
-        <v>29</v>
+        <v>106</v>
       </c>
       <c r="E982" s="8">
-        <v>10098.741248</v>
+        <v>1549098.287104</v>
       </c>
       <c r="F982" s="9">
-        <v>20.477195149346</v>
+        <v>27.26877121915166</v>
       </c>
       <c r="G982" s="9">
-        <v>16.54853951890034</v>
+        <v>17.17879328340446</v>
       </c>
       <c r="H982" s="9">
-        <v>15.94916966003723</v>
+        <v>-3.63716543141238</v>
       </c>
       <c r="I982" s="9">
-        <v>21.42672873942377</v>
+        <v>27.48178207412952</v>
       </c>
       <c r="J982" s="11">
-        <v>17.95710263675431</v>
+        <v>14.22299607097575</v>
       </c>
       <c r="K982" s="9">
-        <v>1.82609388112129</v>
+        <v>1.64987913838446</v>
       </c>
       <c r="L982" s="9">
-        <v>21.4</v>
+        <v>33.1</v>
       </c>
       <c r="M982" s="7" t="s">
-        <v>256</v>
+        <v>2006</v>
       </c>
       <c r="N982" s="9">
-        <v>20.39838349932646</v>
+        <v>29.42524549536546</v>
       </c>
       <c r="O982" s="7" t="s">
-        <v>2477</v>
+        <v>401</v>
       </c>
       <c r="P982" s="9">
-        <v>17.12488350419385</v>
+        <v>50.05807200929154</v>
       </c>
       <c r="Q982" s="9">
-        <v>0.4816441383707154</v>
+        <v>0.9137508085080848</v>
       </c>
       <c r="R982" s="7" t="s">
         <v>46</v>
       </c>
       <c r="S982" s="9">
-        <v>6.833357346207379</v>
+        <v>19.1781681298909</v>
       </c>
       <c r="T982" s="10" t="s">
         <v>30</v>
@@ -71463,63 +71421,63 @@
         <v>30</v>
       </c>
       <c r="V982" s="11">
-        <v>74.52087794432549</v>
+        <v>77.56263383297643</v>
       </c>
     </row>
     <row r="983" spans="1:22">
       <c r="A983" s="6" t="s">
-        <v>2478</v>
+        <v>2473</v>
       </c>
       <c r="B983" s="7" t="s">
-        <v>2479</v>
+        <v>2474</v>
       </c>
       <c r="C983" s="7" t="s">
-        <v>28</v>
+        <v>431</v>
       </c>
       <c r="D983" s="7" t="s">
-        <v>29</v>
+        <v>59</v>
       </c>
       <c r="E983" s="8">
-        <v>147615.596544</v>
-      </c>
-      <c r="F983" s="9">
-        <v>15.94268540560896</v>
-      </c>
-      <c r="G983" s="9">
-        <v>1.19662953118814</v>
+        <v>117310.226432</v>
+      </c>
+      <c r="F983" s="10" t="s">
+        <v>30</v>
+      </c>
+      <c r="G983" s="10" t="s">
+        <v>30</v>
       </c>
       <c r="H983" s="10" t="s">
         <v>30</v>
       </c>
-      <c r="I983" s="9">
-        <v>18.39474460776682</v>
+      <c r="I983" s="10" t="s">
+        <v>30</v>
       </c>
       <c r="J983" s="11">
-        <v>7.826613960296955</v>
+        <v>7.661885357875487</v>
       </c>
       <c r="K983" s="9">
-        <v>8.384361437248861</v>
+        <v>4.31857047257225</v>
       </c>
       <c r="L983" s="9">
-        <v>5.4</v>
-      </c>
-      <c r="M983" s="7" t="s">
-        <v>2480</v>
-      </c>
-      <c r="N983" s="9">
-        <v>18.86635609511109</v>
-      </c>
-      <c r="O983" s="7" t="s">
-        <v>2481</v>
-      </c>
-      <c r="P983" s="9">
-        <v>128.5714285714286</v>
-      </c>
-      <c r="Q983" s="9">
-        <v>1.895410792529631</v>
-      </c>
-      <c r="R983" s="7" t="s">
-        <v>52</v>
+        <v>15.6</v>
+      </c>
+      <c r="M983" s="10" t="s">
+        <v>30</v>
+      </c>
+      <c r="N983" s="10" t="s">
+        <v>30</v>
+      </c>
+      <c r="O983" s="10" t="s">
+        <v>30</v>
+      </c>
+      <c r="P983" s="10" t="s">
+        <v>30</v>
+      </c>
+      <c r="Q983" s="10" t="s">
+        <v>30</v>
+      </c>
+      <c r="R983" s="10" t="s">
+        <v>30</v>
       </c>
       <c r="S983" s="10" t="s">
         <v>30</v>
@@ -71531,66 +71489,66 @@
         <v>30</v>
       </c>
       <c r="V983" s="11">
-        <v>88.94245182012848</v>
+        <v>87.10519271948608</v>
       </c>
     </row>
     <row r="984" spans="1:22">
       <c r="A984" s="6" t="s">
-        <v>2482</v>
+        <v>1429</v>
       </c>
       <c r="B984" s="7" t="s">
-        <v>2483</v>
+        <v>2475</v>
       </c>
       <c r="C984" s="7" t="s">
-        <v>620</v>
+        <v>28</v>
       </c>
       <c r="D984" s="7" t="s">
-        <v>49</v>
+        <v>29</v>
       </c>
       <c r="E984" s="8">
-        <v>1175.433984</v>
-      </c>
-      <c r="F984" s="10" t="s">
-        <v>30</v>
-      </c>
-      <c r="G984" s="10" t="s">
-        <v>30</v>
-      </c>
-      <c r="H984" s="10" t="s">
-        <v>30</v>
-      </c>
-      <c r="I984" s="10" t="s">
-        <v>30</v>
+        <v>13737.530368</v>
+      </c>
+      <c r="F984" s="9">
+        <v>22.70878427501843</v>
+      </c>
+      <c r="G984" s="9">
+        <v>19.44603562228006</v>
+      </c>
+      <c r="H984" s="9">
+        <v>6.887117924925961</v>
+      </c>
+      <c r="I984" s="9">
+        <v>9.297987617174019</v>
       </c>
       <c r="J984" s="11">
-        <v>13.35091224105461</v>
-      </c>
-      <c r="K984" s="10" t="s">
-        <v>30</v>
+        <v>34.29916682554814</v>
+      </c>
+      <c r="K984" s="9">
+        <v>-0.79763244968136</v>
       </c>
       <c r="L984" s="9">
-        <v>2.7</v>
-      </c>
-      <c r="M984" s="10" t="s">
-        <v>30</v>
-      </c>
-      <c r="N984" s="10" t="s">
-        <v>30</v>
-      </c>
-      <c r="O984" s="10" t="s">
-        <v>30</v>
-      </c>
-      <c r="P984" s="10" t="s">
-        <v>30</v>
-      </c>
-      <c r="Q984" s="10" t="s">
-        <v>30</v>
-      </c>
-      <c r="R984" s="10" t="s">
-        <v>30</v>
-      </c>
-      <c r="S984" s="10" t="s">
-        <v>30</v>
+        <v>30.5</v>
+      </c>
+      <c r="M984" s="7" t="s">
+        <v>256</v>
+      </c>
+      <c r="N984" s="9">
+        <v>21.07988238904674</v>
+      </c>
+      <c r="O984" s="7" t="s">
+        <v>1431</v>
+      </c>
+      <c r="P984" s="9">
+        <v>72.6327227569078</v>
+      </c>
+      <c r="Q984" s="9">
+        <v>8.712708267897144</v>
+      </c>
+      <c r="R984" s="7" t="s">
+        <v>46</v>
+      </c>
+      <c r="S984" s="9">
+        <v>187.5059661147017</v>
       </c>
       <c r="T984" s="10" t="s">
         <v>30</v>
@@ -71599,151 +71557,151 @@
         <v>30</v>
       </c>
       <c r="V984" s="11">
-        <v>64.33377944325483</v>
+        <v>77.20342612419699</v>
       </c>
     </row>
     <row r="985" spans="1:22">
       <c r="A985" s="6" t="s">
-        <v>778</v>
+        <v>1829</v>
       </c>
       <c r="B985" s="7" t="s">
-        <v>779</v>
+        <v>1830</v>
       </c>
       <c r="C985" s="7" t="s">
         <v>28</v>
       </c>
       <c r="D985" s="7" t="s">
-        <v>59</v>
+        <v>29</v>
       </c>
       <c r="E985" s="8">
-        <v>534.154257935852</v>
+        <v>15452.863488</v>
       </c>
       <c r="F985" s="9">
-        <v>23.05551234768749</v>
+        <v>14.40609890391468</v>
       </c>
       <c r="G985" s="9">
-        <v>19.47457747625621</v>
+        <v>10.10694436354289</v>
       </c>
       <c r="H985" s="9">
-        <v>37.07233835745288</v>
+        <v>-0.8635316709933301</v>
       </c>
       <c r="I985" s="9">
-        <v>23.60027064751609</v>
+        <v>15.02294740921002</v>
       </c>
       <c r="J985" s="11">
-        <v>6.023709596476647</v>
-      </c>
-      <c r="K985" s="10" t="s">
-        <v>30</v>
-      </c>
-      <c r="L985" s="10" t="s">
-        <v>30</v>
+        <v>17.61870897015553</v>
+      </c>
+      <c r="K985" s="9">
+        <v>3.39759030685614</v>
+      </c>
+      <c r="L985" s="9">
+        <v>8.9</v>
       </c>
       <c r="M985" s="7" t="s">
-        <v>780</v>
+        <v>44</v>
       </c>
       <c r="N985" s="9">
-        <v>38.52531915082372</v>
+        <v>25.43663233318406</v>
       </c>
       <c r="O985" s="7" t="s">
-        <v>781</v>
+        <v>1831</v>
       </c>
       <c r="P985" s="9">
-        <v>114.9436090225564</v>
+        <v>15.20092735703247</v>
       </c>
       <c r="Q985" s="9">
-        <v>0.3878347631318946</v>
+        <v>3.907483599359118</v>
       </c>
       <c r="R985" s="7" t="s">
         <v>46</v>
       </c>
       <c r="S985" s="9">
-        <v>-1.15935796408976</v>
-      </c>
-      <c r="T985" s="12" t="s">
-        <v>41</v>
-      </c>
-      <c r="U985" s="12" t="s">
-        <v>41</v>
+        <v>15.2786123366391</v>
+      </c>
+      <c r="T985" s="10" t="s">
+        <v>30</v>
+      </c>
+      <c r="U985" s="10" t="s">
+        <v>30</v>
       </c>
       <c r="V985" s="11">
-        <v>75.28640256959315</v>
+        <v>39.56370449678801</v>
       </c>
     </row>
     <row r="986" spans="1:22">
       <c r="A986" s="6" t="s">
-        <v>2484</v>
+        <v>325</v>
       </c>
       <c r="B986" s="7" t="s">
-        <v>2485</v>
+        <v>326</v>
       </c>
       <c r="C986" s="7" t="s">
         <v>28</v>
       </c>
       <c r="D986" s="7" t="s">
-        <v>49</v>
+        <v>29</v>
       </c>
       <c r="E986" s="8">
-        <v>16598.28865870422</v>
+        <v>12360.63232</v>
       </c>
       <c r="F986" s="9">
-        <v>21.53079305137872</v>
+        <v>73.73796759418487</v>
       </c>
       <c r="G986" s="9">
-        <v>16.14584250459642</v>
+        <v>36.3960657302815</v>
       </c>
       <c r="H986" s="9">
-        <v>41.14270959837187</v>
+        <v>200</v>
       </c>
       <c r="I986" s="9">
-        <v>18.39271566857261</v>
+        <v>156.7465978512902</v>
       </c>
       <c r="J986" s="11">
-        <v>10.20649812161575</v>
-      </c>
-      <c r="K986" s="10" t="s">
-        <v>30</v>
-      </c>
-      <c r="L986" s="10" t="s">
-        <v>30</v>
+        <v>20.05709800490741</v>
+      </c>
+      <c r="K986" s="9">
+        <v>3.97017617946587</v>
+      </c>
+      <c r="L986" s="9">
+        <v>26.5</v>
       </c>
       <c r="M986" s="7" t="s">
-        <v>2486</v>
+        <v>327</v>
       </c>
       <c r="N986" s="9">
-        <v>23.67472979927946</v>
+        <v>28.35376468633872</v>
       </c>
       <c r="O986" s="7" t="s">
-        <v>2487</v>
+        <v>166</v>
       </c>
       <c r="P986" s="9">
-        <v>0.6289308176100628</v>
+        <v>62.81718399622329</v>
       </c>
       <c r="Q986" s="9">
-        <v>1.202120236842841</v>
+        <v>7.54196831711613</v>
       </c>
       <c r="R986" s="7" t="s">
-        <v>46</v>
-      </c>
-      <c r="S986" s="10" t="s">
-        <v>30</v>
-      </c>
-      <c r="T986" s="12" t="s">
-        <v>41</v>
-      </c>
-      <c r="U986" s="12" t="s">
-        <v>41</v>
+        <v>52</v>
+      </c>
+      <c r="S986" s="9">
+        <v>-6.179504129237912</v>
+      </c>
+      <c r="T986" s="10" t="s">
+        <v>30</v>
+      </c>
+      <c r="U986" s="10" t="s">
+        <v>30</v>
       </c>
       <c r="V986" s="11">
-        <v>76.63543897216273</v>
+        <v>68.06316916488223</v>
       </c>
     </row>
     <row r="987" spans="1:22">
       <c r="A987" s="6" t="s">
-        <v>1242</v>
+        <v>1736</v>
       </c>
       <c r="B987" s="7" t="s">
-        <v>1243</v>
+        <v>1737</v>
       </c>
       <c r="C987" s="7" t="s">
         <v>28</v>
@@ -71752,66 +71710,66 @@
         <v>29</v>
       </c>
       <c r="E987" s="8">
-        <v>86041.427968</v>
+        <v>12465.329152</v>
       </c>
       <c r="F987" s="9">
-        <v>-22.76937883819234</v>
+        <v>18.3357672256623</v>
       </c>
       <c r="G987" s="9">
-        <v>-61.74195098692925</v>
+        <v>11.34875053232618</v>
       </c>
       <c r="H987" s="9">
-        <v>200</v>
+        <v>162.6826764963662</v>
       </c>
       <c r="I987" s="9">
-        <v>-52.32238133357679</v>
+        <v>24.64990259395278</v>
       </c>
       <c r="J987" s="11">
-        <v>373.5170470572995</v>
+        <v>11.7959601299469</v>
       </c>
       <c r="K987" s="9">
-        <v>0.3085969797</v>
+        <v>4.39559184774585</v>
       </c>
       <c r="L987" s="9">
-        <v>130.4</v>
+        <v>12.7</v>
       </c>
       <c r="M987" s="7" t="s">
-        <v>1186</v>
+        <v>1738</v>
       </c>
       <c r="N987" s="9">
-        <v>52.91868502365007</v>
+        <v>24.41986345619947</v>
       </c>
       <c r="O987" s="7" t="s">
-        <v>470</v>
+        <v>2476</v>
       </c>
       <c r="P987" s="9">
-        <v>163.4464651714993</v>
+        <v>22.48766554141781</v>
       </c>
       <c r="Q987" s="9">
-        <v>12.2696971103034</v>
+        <v>11.57935981187805</v>
       </c>
       <c r="R987" s="7" t="s">
-        <v>46</v>
+        <v>52</v>
       </c>
       <c r="S987" s="9">
-        <v>22.10992696590466</v>
+        <v>30557.33041489141</v>
       </c>
       <c r="T987" s="12" t="s">
         <v>41</v>
       </c>
-      <c r="U987" s="12" t="s">
-        <v>41</v>
+      <c r="U987" s="10" t="s">
+        <v>30</v>
       </c>
       <c r="V987" s="11">
-        <v>75.28827623126338</v>
+        <v>45.06932548179872</v>
       </c>
     </row>
     <row r="988" spans="1:22">
       <c r="A988" s="6" t="s">
-        <v>2488</v>
+        <v>2477</v>
       </c>
       <c r="B988" s="7" t="s">
-        <v>2489</v>
+        <v>2478</v>
       </c>
       <c r="C988" s="7" t="s">
         <v>28</v>
@@ -71820,46 +71778,46 @@
         <v>29</v>
       </c>
       <c r="E988" s="8">
-        <v>10411.935744</v>
+        <v>147615.596544</v>
       </c>
       <c r="F988" s="9">
-        <v>7.49516988342678</v>
+        <v>15.94268540560896</v>
       </c>
       <c r="G988" s="9">
-        <v>5.433517399693049</v>
-      </c>
-      <c r="H988" s="9">
-        <v>200</v>
+        <v>1.19662953118814</v>
+      </c>
+      <c r="H988" s="10" t="s">
+        <v>30</v>
       </c>
       <c r="I988" s="9">
-        <v>21.17194829228418</v>
+        <v>18.39474460776682</v>
       </c>
       <c r="J988" s="11">
-        <v>9.194940017024711</v>
+        <v>7.826613960296955</v>
       </c>
       <c r="K988" s="9">
-        <v>2.72871941381047</v>
+        <v>8.384361437248861</v>
       </c>
       <c r="L988" s="9">
-        <v>9</v>
+        <v>5.4</v>
       </c>
       <c r="M988" s="7" t="s">
-        <v>2490</v>
+        <v>2479</v>
       </c>
       <c r="N988" s="9">
-        <v>33.33333333333333</v>
+        <v>18.86635609511109</v>
       </c>
       <c r="O988" s="7" t="s">
-        <v>1421</v>
+        <v>2480</v>
       </c>
       <c r="P988" s="9">
-        <v>29.95391705069124</v>
+        <v>128.5714285714286</v>
       </c>
       <c r="Q988" s="9">
-        <v>0.1461085646552368</v>
-      </c>
-      <c r="R988" s="10" t="s">
-        <v>30</v>
+        <v>1.895410792529631</v>
+      </c>
+      <c r="R988" s="7" t="s">
+        <v>52</v>
       </c>
       <c r="S988" s="10" t="s">
         <v>30</v>
@@ -71871,131 +71829,131 @@
         <v>30</v>
       </c>
       <c r="V988" s="11">
-        <v>89.89079229122056</v>
+        <v>88.94245182012848</v>
       </c>
     </row>
     <row r="989" spans="1:22">
       <c r="A989" s="6" t="s">
-        <v>751</v>
+        <v>2481</v>
       </c>
       <c r="B989" s="7" t="s">
-        <v>752</v>
+        <v>2482</v>
       </c>
       <c r="C989" s="7" t="s">
         <v>28</v>
       </c>
       <c r="D989" s="7" t="s">
-        <v>49</v>
+        <v>29</v>
       </c>
       <c r="E989" s="8">
-        <v>2926.623191579819</v>
+        <v>15756.182528</v>
       </c>
       <c r="F989" s="9">
-        <v>8.990214670930561</v>
+        <v>17.10413168579105</v>
       </c>
       <c r="G989" s="9">
-        <v>0.8193503242969901</v>
+        <v>10.90675747723766</v>
       </c>
       <c r="H989" s="9">
-        <v>109.0641279681346</v>
+        <v>10.58118615531343</v>
       </c>
       <c r="I989" s="9">
-        <v>17.44300098669742</v>
+        <v>23.25626384143405</v>
       </c>
       <c r="J989" s="11">
-        <v>8.135008743252369</v>
-      </c>
-      <c r="K989" s="10" t="s">
-        <v>30</v>
-      </c>
-      <c r="L989" s="10" t="s">
-        <v>30</v>
+        <v>17.98634153029206</v>
+      </c>
+      <c r="K989" s="9">
+        <v>3.74805264505247</v>
+      </c>
+      <c r="L989" s="9">
+        <v>42.2</v>
       </c>
       <c r="M989" s="7" t="s">
-        <v>753</v>
+        <v>833</v>
       </c>
       <c r="N989" s="9">
-        <v>25</v>
+        <v>49.53504632057333</v>
       </c>
       <c r="O989" s="7" t="s">
-        <v>754</v>
+        <v>2483</v>
       </c>
       <c r="P989" s="9">
-        <v>166.3685825085373</v>
+        <v>17617.64705882353</v>
       </c>
       <c r="Q989" s="9">
-        <v>2.892338671864557</v>
+        <v>16.47126241409279</v>
       </c>
       <c r="R989" s="7" t="s">
-        <v>52</v>
+        <v>268</v>
       </c>
       <c r="S989" s="9">
-        <v>4.245780791290596</v>
+        <v>-15.51812380815701</v>
       </c>
       <c r="T989" s="10" t="s">
         <v>30</v>
       </c>
-      <c r="U989" s="10" t="s">
-        <v>30</v>
+      <c r="U989" s="12" t="s">
+        <v>41</v>
       </c>
       <c r="V989" s="11">
-        <v>53.18870449678801</v>
+        <v>75.96359743040685</v>
       </c>
     </row>
     <row r="990" spans="1:22">
       <c r="A990" s="6" t="s">
-        <v>2491</v>
+        <v>352</v>
       </c>
       <c r="B990" s="7" t="s">
-        <v>2492</v>
+        <v>353</v>
       </c>
       <c r="C990" s="7" t="s">
         <v>28</v>
       </c>
       <c r="D990" s="7" t="s">
-        <v>29</v>
+        <v>307</v>
       </c>
       <c r="E990" s="8">
-        <v>9583.85152</v>
+        <v>139.989664</v>
       </c>
       <c r="F990" s="9">
-        <v>14.76466103126517</v>
+        <v>68.97923279422618</v>
       </c>
       <c r="G990" s="9">
-        <v>9.339073736097459</v>
-      </c>
-      <c r="H990" s="9">
-        <v>38.10949529512403</v>
-      </c>
-      <c r="I990" s="10" t="s">
-        <v>30</v>
+        <v>-6.563535963905689</v>
+      </c>
+      <c r="H990" s="10" t="s">
+        <v>30</v>
+      </c>
+      <c r="I990" s="9">
+        <v>94.56183874333236</v>
       </c>
       <c r="J990" s="11">
-        <v>7.119610978040907</v>
+        <v>3.225931242158093</v>
       </c>
       <c r="K990" s="9">
-        <v>22.39222403979814</v>
+        <v>3.15112550023693</v>
       </c>
       <c r="L990" s="9">
-        <v>13.5</v>
-      </c>
-      <c r="M990" s="7" t="s">
-        <v>81</v>
-      </c>
-      <c r="N990" s="9">
-        <v>100</v>
-      </c>
-      <c r="O990" s="7" t="s">
-        <v>81</v>
-      </c>
-      <c r="P990" s="9">
-        <v>-26.19047619047618</v>
-      </c>
-      <c r="Q990" s="9">
-        <v>0</v>
-      </c>
-      <c r="R990" s="10" t="s">
-        <v>30</v>
+        <v>-34.3</v>
+      </c>
+      <c r="M990" s="10" t="s">
+        <v>30</v>
+      </c>
+      <c r="N990" s="10" t="s">
+        <v>30</v>
+      </c>
+      <c r="O990" s="10" t="s">
+        <v>30</v>
+      </c>
+      <c r="P990" s="10" t="s">
+        <v>30</v>
+      </c>
+      <c r="Q990" s="10" t="s">
+        <v>30</v>
+      </c>
+      <c r="R990" s="7" t="s">
+        <v>46</v>
       </c>
       <c r="S990" s="10" t="s">
         <v>30</v>
@@ -72007,66 +71965,66 @@
         <v>30</v>
       </c>
       <c r="V990" s="11">
-        <v>63.61509635974304</v>
+        <v>66.00669164882227</v>
       </c>
     </row>
     <row r="991" spans="1:22">
       <c r="A991" s="6" t="s">
-        <v>762</v>
+        <v>2484</v>
       </c>
       <c r="B991" s="7" t="s">
-        <v>763</v>
+        <v>2485</v>
       </c>
       <c r="C991" s="7" t="s">
-        <v>28</v>
+        <v>431</v>
       </c>
       <c r="D991" s="7" t="s">
-        <v>29</v>
+        <v>307</v>
       </c>
       <c r="E991" s="8">
-        <v>28606.16704</v>
-      </c>
-      <c r="F991" s="9">
-        <v>23.02210928808162</v>
-      </c>
-      <c r="G991" s="9">
-        <v>12.3513454013088</v>
-      </c>
-      <c r="H991" s="9">
-        <v>-3155.200934579439</v>
-      </c>
-      <c r="I991" s="9">
-        <v>26.3762128130752</v>
+        <v>7860.636672</v>
+      </c>
+      <c r="F991" s="10" t="s">
+        <v>30</v>
+      </c>
+      <c r="G991" s="10" t="s">
+        <v>30</v>
+      </c>
+      <c r="H991" s="10" t="s">
+        <v>30</v>
+      </c>
+      <c r="I991" s="10" t="s">
+        <v>30</v>
       </c>
       <c r="J991" s="11">
-        <v>8.784983736132059</v>
+        <v>0.3665657232603735</v>
       </c>
       <c r="K991" s="9">
-        <v>6.69781258468104</v>
+        <v>9.900597324033141</v>
       </c>
       <c r="L991" s="9">
-        <v>1.9</v>
-      </c>
-      <c r="M991" s="7" t="s">
-        <v>764</v>
-      </c>
-      <c r="N991" s="9">
-        <v>24.8367335547431</v>
-      </c>
-      <c r="O991" s="7" t="s">
-        <v>765</v>
-      </c>
-      <c r="P991" s="9">
-        <v>196.661101836394</v>
-      </c>
-      <c r="Q991" s="9">
-        <v>0.5986147521012869</v>
-      </c>
-      <c r="R991" s="7" t="s">
-        <v>268</v>
-      </c>
-      <c r="S991" s="9">
-        <v>-5.323343713571752</v>
+        <v>3.1</v>
+      </c>
+      <c r="M991" s="10" t="s">
+        <v>30</v>
+      </c>
+      <c r="N991" s="10" t="s">
+        <v>30</v>
+      </c>
+      <c r="O991" s="10" t="s">
+        <v>30</v>
+      </c>
+      <c r="P991" s="10" t="s">
+        <v>30</v>
+      </c>
+      <c r="Q991" s="10" t="s">
+        <v>30</v>
+      </c>
+      <c r="R991" s="10" t="s">
+        <v>30</v>
+      </c>
+      <c r="S991" s="10" t="s">
+        <v>30</v>
       </c>
       <c r="T991" s="10" t="s">
         <v>30</v>
@@ -72075,66 +72033,66 @@
         <v>30</v>
       </c>
       <c r="V991" s="11">
-        <v>82.39400428265525</v>
+        <v>71.8953426124197</v>
       </c>
     </row>
     <row r="992" spans="1:22">
       <c r="A992" s="6" t="s">
-        <v>2493</v>
+        <v>2025</v>
       </c>
       <c r="B992" s="7" t="s">
-        <v>2494</v>
+        <v>2026</v>
       </c>
       <c r="C992" s="7" t="s">
         <v>28</v>
       </c>
       <c r="D992" s="7" t="s">
-        <v>106</v>
+        <v>29</v>
       </c>
       <c r="E992" s="8">
-        <v>316416.196608</v>
+        <v>100520.255488</v>
       </c>
       <c r="F992" s="9">
-        <v>7.105064761849279</v>
+        <v>19.74290983466965</v>
       </c>
       <c r="G992" s="9">
-        <v>5.982680344439021</v>
+        <v>2.85946953226829</v>
       </c>
       <c r="H992" s="9">
-        <v>8.718370604228911</v>
+        <v>-1.14691627188177</v>
       </c>
       <c r="I992" s="9">
-        <v>11.96801965473218</v>
+        <v>27.15547778263739</v>
       </c>
       <c r="J992" s="11">
-        <v>29.6417692182084</v>
+        <v>67.60467140210618</v>
       </c>
       <c r="K992" s="9">
-        <v>1.79131150831129</v>
+        <v>3.08019756711583</v>
       </c>
       <c r="L992" s="9">
-        <v>24.7</v>
+        <v>65.5</v>
       </c>
       <c r="M992" s="7" t="s">
-        <v>2495</v>
+        <v>2027</v>
       </c>
       <c r="N992" s="9">
-        <v>27.31445406924166</v>
+        <v>25.05531709954961</v>
       </c>
       <c r="O992" s="7" t="s">
-        <v>45</v>
+        <v>1066</v>
       </c>
       <c r="P992" s="9">
-        <v>49.49564736769378</v>
+        <v>44.57323978496024</v>
       </c>
       <c r="Q992" s="9">
-        <v>3.371631767229602</v>
+        <v>2.092357279705445</v>
       </c>
       <c r="R992" s="7" t="s">
         <v>52</v>
       </c>
       <c r="S992" s="9">
-        <v>30.61461997847589</v>
+        <v>25.02212629438111</v>
       </c>
       <c r="T992" s="10" t="s">
         <v>30</v>
@@ -72143,66 +72101,66 @@
         <v>30</v>
       </c>
       <c r="V992" s="11">
-        <v>80.95503211991435</v>
+        <v>86.09823340471091</v>
       </c>
     </row>
     <row r="993" spans="1:22">
       <c r="A993" s="6" t="s">
-        <v>2496</v>
+        <v>120</v>
       </c>
       <c r="B993" s="7" t="s">
-        <v>2497</v>
+        <v>121</v>
       </c>
       <c r="C993" s="7" t="s">
         <v>28</v>
       </c>
       <c r="D993" s="7" t="s">
-        <v>29</v>
+        <v>106</v>
       </c>
       <c r="E993" s="8">
-        <v>39015.5264</v>
+        <v>343117.49632</v>
       </c>
       <c r="F993" s="9">
-        <v>17.42239589095219</v>
+        <v>56.16048279606593</v>
       </c>
       <c r="G993" s="9">
-        <v>12.03354799162836</v>
+        <v>45.03073679491686</v>
       </c>
       <c r="H993" s="9">
-        <v>200</v>
+        <v>-44.74109110086793</v>
       </c>
       <c r="I993" s="9">
-        <v>23.0751023443879</v>
+        <v>58.23011867639675</v>
       </c>
       <c r="J993" s="11">
-        <v>6.290858837118098</v>
+        <v>36.88889522486986</v>
       </c>
       <c r="K993" s="9">
-        <v>10.4663461159914</v>
+        <v>0.8861031782431901</v>
       </c>
       <c r="L993" s="9">
-        <v>7.199999999999999</v>
+        <v>11.4</v>
       </c>
       <c r="M993" s="7" t="s">
-        <v>2498</v>
+        <v>122</v>
       </c>
       <c r="N993" s="9">
-        <v>44.91438562643193</v>
+        <v>46.22234535164444</v>
       </c>
       <c r="O993" s="7" t="s">
-        <v>2499</v>
+        <v>123</v>
       </c>
       <c r="P993" s="9">
-        <v>14.17935702199662</v>
+        <v>50.52770448548814</v>
       </c>
       <c r="Q993" s="9">
-        <v>9.664266463869753</v>
-      </c>
-      <c r="R993" s="10" t="s">
-        <v>30</v>
-      </c>
-      <c r="S993" s="10" t="s">
-        <v>30</v>
+        <v>5.238834997307484</v>
+      </c>
+      <c r="R993" s="7" t="s">
+        <v>46</v>
+      </c>
+      <c r="S993" s="9">
+        <v>13.62692432441163</v>
       </c>
       <c r="T993" s="10" t="s">
         <v>30</v>
@@ -72211,15 +72169,15 @@
         <v>30</v>
       </c>
       <c r="V993" s="11">
-        <v>41.95931477516059</v>
+        <v>41.9710920770878</v>
       </c>
     </row>
     <row r="994" spans="1:22">
       <c r="A994" s="6" t="s">
-        <v>902</v>
+        <v>2486</v>
       </c>
       <c r="B994" s="7" t="s">
-        <v>903</v>
+        <v>2487</v>
       </c>
       <c r="C994" s="7" t="s">
         <v>28</v>
@@ -72228,194 +72186,194 @@
         <v>29</v>
       </c>
       <c r="E994" s="8">
-        <v>16507.032576</v>
+        <v>22208.309248</v>
       </c>
       <c r="F994" s="9">
-        <v>15.58608160554067</v>
+        <v>21.31256916296736</v>
       </c>
       <c r="G994" s="9">
-        <v>6.58630328441649</v>
+        <v>15.70131812244106</v>
       </c>
       <c r="H994" s="9">
-        <v>-22.15173053427627</v>
+        <v>61.85351566119409</v>
       </c>
       <c r="I994" s="9">
-        <v>12.05096674017734</v>
+        <v>31.15588367065784</v>
       </c>
       <c r="J994" s="11">
-        <v>5.530745092896175</v>
+        <v>23.28198974227121</v>
       </c>
       <c r="K994" s="9">
-        <v>5.30455743616265</v>
+        <v>3.41846161957767</v>
       </c>
       <c r="L994" s="9">
-        <v>8.5</v>
+        <v>11</v>
       </c>
       <c r="M994" s="7" t="s">
-        <v>2500</v>
+        <v>2488</v>
       </c>
       <c r="N994" s="9">
-        <v>63.40903066183618</v>
+        <v>35.82748302678579</v>
       </c>
       <c r="O994" s="7" t="s">
-        <v>2501</v>
+        <v>332</v>
       </c>
       <c r="P994" s="9">
-        <v>12600</v>
+        <v>12.09423821395907</v>
       </c>
       <c r="Q994" s="9">
-        <v>8.897851712612685</v>
+        <v>0.2649807808230181</v>
       </c>
       <c r="R994" s="7" t="s">
         <v>52</v>
       </c>
-      <c r="S994" s="10" t="s">
-        <v>30</v>
+      <c r="S994" s="9">
+        <v>2.192982456140358</v>
       </c>
       <c r="T994" s="10" t="s">
         <v>30</v>
       </c>
-      <c r="U994" s="12" t="s">
-        <v>41</v>
+      <c r="U994" s="10" t="s">
+        <v>30</v>
       </c>
       <c r="V994" s="11">
-        <v>90.01043897216273</v>
+        <v>72.3661670235546</v>
       </c>
     </row>
     <row r="995" spans="1:22">
       <c r="A995" s="6" t="s">
-        <v>2502</v>
+        <v>937</v>
       </c>
       <c r="B995" s="7" t="s">
-        <v>2503</v>
+        <v>938</v>
       </c>
       <c r="C995" s="7" t="s">
-        <v>431</v>
+        <v>28</v>
       </c>
       <c r="D995" s="7" t="s">
-        <v>307</v>
+        <v>29</v>
       </c>
       <c r="E995" s="8">
-        <v>13979.88864</v>
-      </c>
-      <c r="F995" s="10" t="s">
-        <v>30</v>
-      </c>
-      <c r="G995" s="10" t="s">
-        <v>30</v>
-      </c>
-      <c r="H995" s="10" t="s">
-        <v>30</v>
-      </c>
-      <c r="I995" s="10" t="s">
-        <v>30</v>
+        <v>12343.648256</v>
+      </c>
+      <c r="F995" s="9">
+        <v>16.32630569798057</v>
+      </c>
+      <c r="G995" s="9">
+        <v>8.34937966664376</v>
+      </c>
+      <c r="H995" s="9">
+        <v>200</v>
+      </c>
+      <c r="I995" s="9">
+        <v>14.92643595649632</v>
       </c>
       <c r="J995" s="11">
-        <v>5.149601967536442</v>
+        <v>20.48611105504418</v>
       </c>
       <c r="K995" s="9">
-        <v>-13.5739633473933</v>
+        <v>2.23980692147162</v>
       </c>
       <c r="L995" s="9">
-        <v>7.5</v>
-      </c>
-      <c r="M995" s="10" t="s">
-        <v>30</v>
-      </c>
-      <c r="N995" s="10" t="s">
-        <v>30</v>
-      </c>
-      <c r="O995" s="10" t="s">
-        <v>30</v>
-      </c>
-      <c r="P995" s="10" t="s">
-        <v>30</v>
-      </c>
-      <c r="Q995" s="10" t="s">
-        <v>30</v>
-      </c>
-      <c r="R995" s="10" t="s">
-        <v>30</v>
-      </c>
-      <c r="S995" s="10" t="s">
-        <v>30</v>
-      </c>
-      <c r="T995" s="10" t="s">
-        <v>30</v>
-      </c>
-      <c r="U995" s="10" t="s">
-        <v>30</v>
+        <v>34.4</v>
+      </c>
+      <c r="M995" s="7" t="s">
+        <v>939</v>
+      </c>
+      <c r="N995" s="9">
+        <v>33.33333333333333</v>
+      </c>
+      <c r="O995" s="7" t="s">
+        <v>939</v>
+      </c>
+      <c r="P995" s="9">
+        <v>3948.102189781021</v>
+      </c>
+      <c r="Q995" s="9">
+        <v>31.90432977647047</v>
+      </c>
+      <c r="R995" s="7" t="s">
+        <v>46</v>
+      </c>
+      <c r="S995" s="9">
+        <v>31.73373240736936</v>
+      </c>
+      <c r="T995" s="12" t="s">
+        <v>41</v>
+      </c>
+      <c r="U995" s="12" t="s">
+        <v>41</v>
       </c>
       <c r="V995" s="11">
-        <v>75.90497858672377</v>
+        <v>44.03078158458244</v>
       </c>
     </row>
     <row r="996" spans="1:22">
       <c r="A996" s="6" t="s">
-        <v>1887</v>
+        <v>2489</v>
       </c>
       <c r="B996" s="7" t="s">
-        <v>2504</v>
+        <v>2490</v>
       </c>
       <c r="C996" s="7" t="s">
         <v>28</v>
       </c>
       <c r="D996" s="7" t="s">
-        <v>29</v>
+        <v>59</v>
       </c>
       <c r="E996" s="8">
-        <v>58120.298496</v>
+        <v>709.240768</v>
       </c>
       <c r="F996" s="9">
-        <v>8.10095776525935</v>
+        <v>10.67763396984633</v>
       </c>
       <c r="G996" s="9">
-        <v>5.32340163435406</v>
-      </c>
-      <c r="H996" s="10" t="s">
-        <v>30</v>
+        <v>7.02173275861261</v>
+      </c>
+      <c r="H996" s="9">
+        <v>-329.46879962913</v>
       </c>
       <c r="I996" s="9">
-        <v>11.49500056642986</v>
+        <v>10.5115828482743</v>
       </c>
       <c r="J996" s="11">
-        <v>30.31001799813607</v>
-      </c>
-      <c r="K996" s="10" t="s">
-        <v>30</v>
+        <v>7.821643636363636</v>
+      </c>
+      <c r="K996" s="9">
+        <v>8.540823191934729</v>
       </c>
       <c r="L996" s="9">
-        <v>190</v>
+        <v>5.800000000000001</v>
       </c>
       <c r="M996" s="7" t="s">
-        <v>28</v>
+        <v>1643</v>
       </c>
       <c r="N996" s="9">
-        <v>32.70637408568443</v>
+        <v>77.68604388147477</v>
       </c>
       <c r="O996" s="7" t="s">
-        <v>1889</v>
+        <v>1788</v>
       </c>
       <c r="P996" s="9">
-        <v>12.88696904247659</v>
+        <v>6.995661605206083</v>
       </c>
       <c r="Q996" s="9">
-        <v>18.57941017706166</v>
+        <v>3.181355994018062</v>
       </c>
       <c r="R996" s="7" t="s">
         <v>52</v>
       </c>
-      <c r="S996" s="9">
-        <v>11.10354778258158</v>
+      <c r="S996" s="10" t="s">
+        <v>30</v>
       </c>
       <c r="T996" s="10" t="s">
         <v>30</v>
       </c>
-      <c r="U996" s="12" t="s">
-        <v>41</v>
+      <c r="U996" s="10" t="s">
+        <v>30</v>
       </c>
       <c r="V996" s="11">
-        <v>81.39105995717344</v>
+        <v>41.40604925053533</v>
       </c>
     </row>
   </sheetData>

</xml_diff>